<commit_message>
Anh: data preprocessing & EDA report
</commit_message>
<xml_diff>
--- a/TLCN_EDA_AQI/EDA_AQI/Jobs/src/eda/eda_reports/openmeteo_2024_eda_report.xlsx
+++ b/TLCN_EDA_AQI/EDA_AQI/Jobs/src/eda/eda_reports/openmeteo_2024_eda_report.xlsx
@@ -697,10 +697,10 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>379.0556175209241</v>
+        <v>379.0558869982246</v>
       </c>
       <c r="G8" t="n">
-        <v>246.8572112033226</v>
+        <v>246.857373798771</v>
       </c>
       <c r="H8" t="n">
         <v>80</v>

</xml_diff>